<commit_message>
Set real author metadata on memo.pdf and dashboard.xlsx
</commit_message>
<xml_diff>
--- a/dashboard/PhonePe_Digital_Payments_Dashboard.xlsx
+++ b/dashboard/PhonePe_Digital_Payments_Dashboard.xlsx
@@ -1511,7 +1511,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>71238642397.16028</v>
+        <v>71238642397.16029</v>
       </c>
       <c r="C3" t="n">
         <v/>
@@ -1577,7 +1577,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>70030598500.48001</v>
+        <v>70030598500.48003</v>
       </c>
       <c r="C9" t="n">
         <v/>
@@ -1643,7 +1643,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>100037360294.7793</v>
+        <v>100037360294.7794</v>
       </c>
       <c r="C15" t="n">
         <v/>
@@ -1665,7 +1665,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>67890541472.40013</v>
+        <v>67890541472.40014</v>
       </c>
       <c r="C17" t="n">
         <v/>
@@ -2086,16 +2086,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1588249</v>
+        <v>1589977</v>
       </c>
       <c r="C11" t="n">
-        <v>540790288428.26</v>
+        <v>542046280325.81</v>
       </c>
       <c r="D11" t="n">
-        <v>25</v>
+        <v>25.03</v>
       </c>
       <c r="E11" t="n">
-        <v>47.26</v>
+        <v>47.37</v>
       </c>
     </row>
     <row r="12">
@@ -2105,16 +2105,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1588404</v>
+        <v>1586676</v>
       </c>
       <c r="C12" t="n">
-        <v>538052422916.15</v>
+        <v>536796431018.6</v>
       </c>
       <c r="D12" t="n">
-        <v>25</v>
+        <v>24.97</v>
       </c>
       <c r="E12" t="n">
-        <v>47.02</v>
+        <v>46.91</v>
       </c>
     </row>
     <row r="13">
@@ -2124,13 +2124,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1588404</v>
+        <v>1586676</v>
       </c>
       <c r="C13" t="n">
-        <v>32783246268.29</v>
+        <v>32759365241.1</v>
       </c>
       <c r="D13" t="n">
-        <v>25</v>
+        <v>24.97</v>
       </c>
       <c r="E13" t="n">
         <v>2.86</v>
@@ -2143,16 +2143,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>792275</v>
+        <v>799323</v>
       </c>
       <c r="C14" t="n">
-        <v>16937343125.8</v>
+        <v>17082504268.23</v>
       </c>
       <c r="D14" t="n">
-        <v>12.47</v>
+        <v>12.58</v>
       </c>
       <c r="E14" t="n">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="15">
@@ -2162,16 +2162,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>795975</v>
+        <v>790655</v>
       </c>
       <c r="C15" t="n">
-        <v>15829644021.27</v>
+        <v>15708363906.03</v>
       </c>
       <c r="D15" t="n">
-        <v>12.53</v>
+        <v>12.44</v>
       </c>
       <c r="E15" t="n">
-        <v>1.38</v>
+        <v>1.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>